<commit_message>
refactor: remove conteúdo opinativo, oculta Expectativa e renomeia aba Ranking
- Remove narrativas subjetivas (buildNarrative, buildTechnicalNarrative, buildLeagueContextNarrative, buildHeadToHeadNarrative) do Por Quadrilha
- Remove card "Expectativa 2026 · Leitura Projetada" e linha de expectativa no grid de quesitos
- Substitui métricas de projeção por ranks históricos reais (rank no grupo / rank na liga)
- Oculta aba Expectativa 2026 (desktop e mobile)
- Renomeia aba "Ranking" para "Desempenho" em toda a interface
- Remove medalhas 🥇🥈🥉 da UI
- Corrige planilhas de notas (acesso-2022, acesso-2023, acesso-2025, especial-2022)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/assets/notas/acesso-2022.xlsx
+++ b/dashboard/assets/notas/acesso-2022.xlsx
@@ -1,266 +1,43 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <Application>Microsoft Excel</Application>
-  <DocSecurity>0</DocSecurity>
-  <ScaleCrop>false</ScaleCrop>
-  <HeadingPairs>
-    <vt:vector size="2" baseType="variant">
-      <vt:variant>
-        <vt:lpstr>Planilhas</vt:lpstr>
-      </vt:variant>
-      <vt:variant>
-        <vt:i4>7</vt:i4>
-      </vt:variant>
-    </vt:vector>
-  </HeadingPairs>
-  <TitlesOfParts>
-    <vt:vector size="7" baseType="lpstr">
-      <vt:lpstr>TOTAL</vt:lpstr>
-      <vt:lpstr>COREOGRAFIA</vt:lpstr>
-      <vt:lpstr>MARCAÇÃO</vt:lpstr>
-      <vt:lpstr>ANIMAÇÃO</vt:lpstr>
-      <vt:lpstr>FIGURINO</vt:lpstr>
-      <vt:lpstr>CASAL DO NOIVOS</vt:lpstr>
-      <vt:lpstr>TRILHA SONORA</vt:lpstr>
-    </vt:vector>
-  </TitlesOfParts>
-  <LinksUpToDate>false</LinksUpToDate>
-  <SharedDoc>false</SharedDoc>
-  <HyperlinksChanged>false</HyperlinksChanged>
-  <AppVersion>16.0300</AppVersion>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24326"/>
+  <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tiago\Documents\GitHub\site-linq-dfe-beta\dashboard\assets\notas\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0B7C7B8-FB62-4F23-B4F6-7417FFE478CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="TOTAL" sheetId="7" r:id="rId1"/>
+    <sheet name="COREOGRAFIA" sheetId="1" r:id="rId2"/>
+    <sheet name="MARCAÇÃO" sheetId="2" r:id="rId3"/>
+    <sheet name="ANIMAÇÃO" sheetId="3" r:id="rId4"/>
+    <sheet name="FIGURINO" sheetId="4" r:id="rId5"/>
+    <sheet name="CASAL DO NOIVOS" sheetId="5" r:id="rId6"/>
+    <sheet name="TRILHA SONORA" sheetId="6" r:id="rId7"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <dc:title>e506e5675554a47eec29531626cec8d946390a733ca6491f5fe1f34c15789cb3.xlsx</dc:title>
-  <dc:creator>Work4</dc:creator>
-  <cp:lastModifiedBy>Tiago</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-12T20:28:07Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-15T11:00:37Z</dcterms:modified>
-</cp:coreProperties>
-</file>
-
-<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2" name="Created">
-    <vt:filetime>2026-03-12T00:00:00Z</vt:filetime>
-  </property>
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="Creator">
-    <vt:lpwstr>EXCEL.EXE</vt:lpwstr>
-  </property>
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="LastSaved">
-    <vt:filetime>2026-03-12T00:00:00Z</vt:filetime>
-  </property>
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="5" name="Producer">
-    <vt:lpwstr>www.ilovepdf.com</vt:lpwstr>
-  </property>
-</Properties>
-</file>
-
-<file path=xl\calcChain.xml><?xml version="1.0" encoding="utf-8"?>
-<calcChain xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <c r="H14" i="6" l="1"/>
-  <c r="I14" i="6" s="1"/>
-  <c r="H14" i="5"/>
-  <c r="I14" i="5" s="1"/>
-  <c r="H14" i="4"/>
-  <c r="I14" i="4" s="1"/>
-  <c r="H14" i="3"/>
-  <c r="I14" i="3" s="1"/>
-  <c r="H14" i="2"/>
-  <c r="H14" i="1"/>
-  <c r="H14" i="7"/>
-  <c r="H13" i="6"/>
-  <c r="I13" i="6" s="1"/>
-  <c r="H12" i="6"/>
-  <c r="I12" i="6" s="1"/>
-  <c r="H11" i="6"/>
-  <c r="I11" i="6" s="1"/>
-  <c r="H10" i="6"/>
-  <c r="I10" i="6" s="1"/>
-  <c r="H9" i="6"/>
-  <c r="I9" i="6" s="1"/>
-  <c r="H8" i="6"/>
-  <c r="I8" i="6" s="1"/>
-  <c r="H7" i="6"/>
-  <c r="I7" i="6" s="1"/>
-  <c r="H6" i="6"/>
-  <c r="I6" i="6" s="1"/>
-  <c r="H5" i="6"/>
-  <c r="I5" i="6" s="1"/>
-  <c r="H4" i="6"/>
-  <c r="I4" i="6" s="1"/>
-  <c r="H3" i="6"/>
-  <c r="I3" i="6" s="1"/>
-  <c r="H2" i="6"/>
-  <c r="I2" i="6" s="1"/>
-  <c r="H13" i="5"/>
-  <c r="I13" i="5" s="1"/>
-  <c r="H12" i="5"/>
-  <c r="I12" i="5" s="1"/>
-  <c r="H11" i="5"/>
-  <c r="I11" i="5" s="1"/>
-  <c r="H10" i="5"/>
-  <c r="I10" i="5" s="1"/>
-  <c r="H9" i="5"/>
-  <c r="I9" i="5" s="1"/>
-  <c r="H8" i="5"/>
-  <c r="I8" i="5" s="1"/>
-  <c r="H7" i="5"/>
-  <c r="I7" i="5" s="1"/>
-  <c r="H6" i="5"/>
-  <c r="I6" i="5" s="1"/>
-  <c r="H5" i="5"/>
-  <c r="I5" i="5" s="1"/>
-  <c r="H4" i="5"/>
-  <c r="I4" i="5" s="1"/>
-  <c r="H3" i="5"/>
-  <c r="I3" i="5" s="1"/>
-  <c r="H2" i="5"/>
-  <c r="I2" i="5" s="1"/>
-  <c r="H13" i="4"/>
-  <c r="I13" i="4" s="1"/>
-  <c r="H12" i="4"/>
-  <c r="I12" i="4" s="1"/>
-  <c r="H11" i="4"/>
-  <c r="I11" i="4" s="1"/>
-  <c r="H10" i="4"/>
-  <c r="I10" i="4" s="1"/>
-  <c r="H9" i="4"/>
-  <c r="I9" i="4" s="1"/>
-  <c r="H8" i="4"/>
-  <c r="I8" i="4" s="1"/>
-  <c r="H7" i="4"/>
-  <c r="I7" i="4" s="1"/>
-  <c r="H6" i="4"/>
-  <c r="I6" i="4" s="1"/>
-  <c r="H5" i="4"/>
-  <c r="I5" i="4" s="1"/>
-  <c r="H4" i="4"/>
-  <c r="I4" i="4" s="1"/>
-  <c r="H3" i="4"/>
-  <c r="I3" i="4" s="1"/>
-  <c r="H2" i="4"/>
-  <c r="I2" i="4" s="1"/>
-  <c r="H13" i="3"/>
-  <c r="I13" i="3" s="1"/>
-  <c r="H12" i="3"/>
-  <c r="I12" i="3" s="1"/>
-  <c r="H11" i="3"/>
-  <c r="I11" i="3" s="1"/>
-  <c r="H10" i="3"/>
-  <c r="I10" i="3" s="1"/>
-  <c r="H9" i="3"/>
-  <c r="I9" i="3" s="1"/>
-  <c r="H8" i="3"/>
-  <c r="I8" i="3" s="1"/>
-  <c r="H7" i="3"/>
-  <c r="I7" i="3" s="1"/>
-  <c r="H6" i="3"/>
-  <c r="I6" i="3" s="1"/>
-  <c r="H5" i="3"/>
-  <c r="I5" i="3" s="1"/>
-  <c r="H4" i="3"/>
-  <c r="I4" i="3" s="1"/>
-  <c r="H3" i="3"/>
-  <c r="I3" i="3" s="1"/>
-  <c r="H2" i="3"/>
-  <c r="I2" i="3" s="1"/>
-  <c r="I14" i="2"/>
-  <c r="H13" i="2"/>
-  <c r="I13" i="2" s="1"/>
-  <c r="H12" i="2"/>
-  <c r="I12" i="2" s="1"/>
-  <c r="H11" i="2"/>
-  <c r="I11" i="2" s="1"/>
-  <c r="H10" i="2"/>
-  <c r="I10" i="2" s="1"/>
-  <c r="H9" i="2"/>
-  <c r="I9" i="2" s="1"/>
-  <c r="H8" i="2"/>
-  <c r="I8" i="2" s="1"/>
-  <c r="H7" i="2"/>
-  <c r="I7" i="2" s="1"/>
-  <c r="H6" i="2"/>
-  <c r="I6" i="2" s="1"/>
-  <c r="H5" i="2"/>
-  <c r="I5" i="2" s="1"/>
-  <c r="H4" i="2"/>
-  <c r="I4" i="2" s="1"/>
-  <c r="H3" i="2"/>
-  <c r="I3" i="2" s="1"/>
-  <c r="H2" i="2"/>
-  <c r="I2" i="2" s="1"/>
-  <c r="H3" i="1"/>
-  <c r="I3" i="1" s="1"/>
-  <c r="H4" i="1"/>
-  <c r="I4" i="1"/>
-  <c r="H5" i="1"/>
-  <c r="I5" i="1" s="1"/>
-  <c r="H6" i="1"/>
-  <c r="I6" i="1" s="1"/>
-  <c r="H7" i="1"/>
-  <c r="I7" i="1" s="1"/>
-  <c r="H8" i="1"/>
-  <c r="I8" i="1" s="1"/>
-  <c r="H9" i="1"/>
-  <c r="I9" i="1" s="1"/>
-  <c r="H10" i="1"/>
-  <c r="I10" i="1" s="1"/>
-  <c r="H11" i="1"/>
-  <c r="I11" i="1"/>
-  <c r="H12" i="1"/>
-  <c r="I12" i="1"/>
-  <c r="H13" i="1"/>
-  <c r="I13" i="1" s="1"/>
-  <c r="I14" i="1"/>
-  <c r="H2" i="1"/>
-  <c r="I2" i="1" s="1"/>
-  <c r="J4" i="7"/>
-  <c r="J6" i="7"/>
-  <c r="J12" i="7"/>
-  <c r="I4" i="7"/>
-  <c r="I5" i="7"/>
-  <c r="J5" i="7" s="1"/>
-  <c r="I6" i="7"/>
-  <c r="I7" i="7"/>
-  <c r="J7" i="7" s="1"/>
-  <c r="I8" i="7"/>
-  <c r="J8" i="7" s="1"/>
-  <c r="I12" i="7"/>
-  <c r="I13" i="7"/>
-  <c r="J13" i="7" s="1"/>
-  <c r="I14" i="7"/>
-  <c r="J14" i="7" s="1"/>
-  <c r="I2" i="7"/>
-  <c r="J2" i="7" s="1"/>
-  <c r="H3" i="7"/>
-  <c r="I3" i="7" s="1"/>
-  <c r="J3" i="7" s="1"/>
-  <c r="H4" i="7"/>
-  <c r="H5" i="7"/>
-  <c r="H6" i="7"/>
-  <c r="H7" i="7"/>
-  <c r="H8" i="7"/>
-  <c r="H9" i="7"/>
-  <c r="I9" i="7" s="1"/>
-  <c r="J9" i="7" s="1"/>
-  <c r="H10" i="7"/>
-  <c r="I10" i="7" s="1"/>
-  <c r="J10" i="7" s="1"/>
-  <c r="H11" i="7"/>
-  <c r="I11" i="7" s="1"/>
-  <c r="J11" i="7" s="1"/>
-  <c r="H12" i="7"/>
-  <c r="H13" i="7"/>
-  <c r="H2" i="7"/>
-</calcChain>
-</file>
-
-<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="29">
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="32">
   <si>
     <r>
       <rPr>
@@ -546,10 +323,19 @@
   <si>
     <t>MÉDIA</t>
   </si>
+  <si>
+    <t>MÉDIA ETAPA</t>
+  </si>
+  <si>
+    <t>MÉDIA CIRCUITO</t>
+  </si>
+  <si>
+    <t>DESCLASSIFICADA</t>
+  </si>
 </sst>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
@@ -642,7 +428,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -715,26 +501,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -745,9 +516,6 @@
       <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -795,23 +563,11 @@
     <xf numFmtId="164" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
@@ -819,8 +575,11 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -839,7 +598,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1158,84 +917,55 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24326"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tiago\Documents\GitHub\fantasy-junino\assets\notas\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F80CCB94-1842-4752-8479-3F48EEA82961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="TOTAL" sheetId="7" r:id="rId1"/>
-    <sheet name="COREOGRAFIA" sheetId="1" r:id="rId2"/>
-    <sheet name="MARCAÇÃO" sheetId="2" r:id="rId3"/>
-    <sheet name="ANIMAÇÃO" sheetId="3" r:id="rId4"/>
-    <sheet name="FIGURINO" sheetId="4" r:id="rId5"/>
-    <sheet name="CASAL DO NOIVOS" sheetId="5" r:id="rId6"/>
-    <sheet name="TRILHA SONORA" sheetId="6" r:id="rId7"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD4F9760-AC26-43DB-A291-7E4EFB740AE9}">
   <dimension ref="A1:J14"/>
   <sheetFormatPr defaultColWidth="27.5" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.5" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.5" style="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="11" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="27.5" style="9"/>
+    <col min="1" max="1" width="3.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="11" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="27.5" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="5"/>
-      <c r="B1" s="6" t="s">
+      <c r="A1" s="4"/>
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="H1" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="11">
+      <c r="A2" s="10">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="11" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="1">
@@ -1251,23 +981,27 @@
         <v>179.6</v>
       </c>
       <c r="G2" s="2">
+        <f>SUM(C2:F2)</f>
         <v>718.2</v>
       </c>
       <c r="H2">
-        <f>G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <f>G2/4</f>
+        <v>179.55</v>
       </c>
       <c r="I2">
-        <f>H2/6</f>
+        <f t="shared" ref="I2:I14" si="0">H2/6</f>
+        <v>29.925000000000001</v>
       </c>
       <c r="J2">
-        <f>I2/3</f>
+        <f t="shared" ref="J2:J14" si="1">I2/3</f>
+        <v>9.9749999999999996</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="11">
+      <c r="A3" s="10">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="1">
@@ -1283,23 +1017,27 @@
         <v>179.6</v>
       </c>
       <c r="G3" s="2">
+        <f t="shared" ref="G3:G14" si="2">SUM(C3:F3)</f>
         <v>714.4</v>
       </c>
       <c r="H3">
-        <f>G3/COUNTIF(C3:F3,"&lt;&gt;0")</f>
+        <f t="shared" ref="H3:H13" si="3">G3/4</f>
+        <v>178.6</v>
       </c>
       <c r="I3">
-        <f>H3/6</f>
+        <f t="shared" si="0"/>
+        <v>29.766666666666666</v>
       </c>
       <c r="J3">
-        <f>I3/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9222222222222225</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="11">
+      <c r="A4" s="10">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="1">
@@ -1315,23 +1053,27 @@
         <v>178.4</v>
       </c>
       <c r="G4" s="2">
+        <f t="shared" si="2"/>
         <v>712.6</v>
       </c>
       <c r="H4">
-        <f>G4/COUNTIF(C4:F4,"&lt;&gt;0")</f>
+        <f t="shared" si="3"/>
+        <v>178.15</v>
       </c>
       <c r="I4">
-        <f>H4/6</f>
+        <f t="shared" si="0"/>
+        <v>29.691666666666666</v>
       </c>
       <c r="J4">
-        <f>I4/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8972222222222221</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="13">
+      <c r="A5" s="12">
         <v>4</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="3">
@@ -1346,24 +1088,28 @@
       <c r="F5" s="3">
         <v>178.6</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="2">
+        <f t="shared" si="2"/>
         <v>712</v>
       </c>
       <c r="H5">
-        <f>G5/COUNTIF(C5:F5,"&lt;&gt;0")</f>
+        <f t="shared" si="3"/>
+        <v>178</v>
       </c>
       <c r="I5">
-        <f>H5/6</f>
+        <f t="shared" si="0"/>
+        <v>29.666666666666668</v>
       </c>
       <c r="J5">
-        <f>I5/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8888888888888893</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="13">
+      <c r="A6" s="12">
         <v>5</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="3">
@@ -1378,24 +1124,28 @@
       <c r="F6" s="3">
         <v>179.4</v>
       </c>
-      <c r="G6" s="4">
-        <v>710.2</v>
+      <c r="G6" s="2">
+        <f t="shared" si="2"/>
+        <v>710.19999999999993</v>
       </c>
       <c r="H6">
-        <f>G6/COUNTIF(C6:F6,"&lt;&gt;0")</f>
+        <f t="shared" si="3"/>
+        <v>177.54999999999998</v>
       </c>
       <c r="I6">
-        <f>H6/6</f>
+        <f t="shared" si="0"/>
+        <v>29.591666666666665</v>
       </c>
       <c r="J6">
-        <f>I6/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8638888888888889</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="13">
+      <c r="A7" s="12">
         <v>6</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="3">
@@ -1410,24 +1160,28 @@
       <c r="F7" s="3">
         <v>179.1</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="2">
+        <f t="shared" si="2"/>
         <v>709.4</v>
       </c>
       <c r="H7">
-        <f>G7/COUNTIF(C7:F7,"&lt;&gt;0")</f>
+        <f t="shared" si="3"/>
+        <v>177.35</v>
       </c>
       <c r="I7">
-        <f>H7/6</f>
+        <f t="shared" si="0"/>
+        <v>29.558333333333334</v>
       </c>
       <c r="J7">
-        <f>I7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8527777777777779</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="13">
+      <c r="A8" s="12">
         <v>7</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="3">
@@ -1442,24 +1196,28 @@
       <c r="F8" s="3">
         <v>178.2</v>
       </c>
-      <c r="G8" s="4">
-        <v>702.1</v>
+      <c r="G8" s="2">
+        <f t="shared" si="2"/>
+        <v>702.09999999999991</v>
       </c>
       <c r="H8">
-        <f>G8/COUNTIF(C8:F8,"&lt;&gt;0")</f>
+        <f t="shared" si="3"/>
+        <v>175.52499999999998</v>
       </c>
       <c r="I8">
-        <f>H8/6</f>
+        <f t="shared" si="0"/>
+        <v>29.254166666666663</v>
       </c>
       <c r="J8">
-        <f>I8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7513888888888882</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="13">
+      <c r="A9" s="12">
         <v>8</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="3">
@@ -1474,24 +1232,28 @@
       <c r="F9" s="3">
         <v>175.2</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="2">
+        <f t="shared" si="2"/>
         <v>699.2</v>
       </c>
       <c r="H9">
-        <f>G9/COUNTIF(C9:F9,"&lt;&gt;0")</f>
+        <f t="shared" si="3"/>
+        <v>174.8</v>
       </c>
       <c r="I9">
-        <f>H9/6</f>
+        <f t="shared" si="0"/>
+        <v>29.133333333333336</v>
       </c>
       <c r="J9">
-        <f>I9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7111111111111121</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="13">
+      <c r="A10" s="12">
         <v>9</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="3">
@@ -1506,24 +1268,28 @@
       <c r="F10" s="3">
         <v>177.7</v>
       </c>
-      <c r="G10" s="4">
-        <v>695.9</v>
+      <c r="G10" s="2">
+        <f t="shared" si="2"/>
+        <v>695.90000000000009</v>
       </c>
       <c r="H10">
-        <f>G10/COUNTIF(C10:F10,"&lt;&gt;0")</f>
+        <f t="shared" si="3"/>
+        <v>173.97500000000002</v>
       </c>
       <c r="I10">
-        <f>H10/6</f>
+        <f t="shared" si="0"/>
+        <v>28.995833333333337</v>
       </c>
       <c r="J10">
-        <f>I10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6652777777777796</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="13">
+      <c r="A11" s="12">
         <v>10</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="3">
@@ -1538,24 +1304,28 @@
       <c r="F11" s="3">
         <v>178.4</v>
       </c>
-      <c r="G11" s="4">
-        <v>692.5</v>
+      <c r="G11" s="2">
+        <f t="shared" si="2"/>
+        <v>692.49999999999989</v>
       </c>
       <c r="H11">
-        <f>G11/COUNTIF(C11:F11,"&lt;&gt;0")</f>
+        <f t="shared" si="3"/>
+        <v>173.12499999999997</v>
       </c>
       <c r="I11">
-        <f>H11/6</f>
+        <f t="shared" si="0"/>
+        <v>28.854166666666661</v>
       </c>
       <c r="J11">
-        <f>I11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6180555555555536</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="13">
+      <c r="A12" s="12">
         <v>11</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="13" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="3">
@@ -1570,24 +1340,28 @@
       <c r="F12" s="3">
         <v>176.4</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="2">
+        <f t="shared" si="2"/>
         <v>686.6</v>
       </c>
       <c r="H12">
-        <f>G12/COUNTIF(C12:F12,"&lt;&gt;0")</f>
+        <f t="shared" si="3"/>
+        <v>171.65</v>
       </c>
       <c r="I12">
-        <f>H12/6</f>
+        <f t="shared" si="0"/>
+        <v>28.608333333333334</v>
       </c>
       <c r="J12">
-        <f>I12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.5361111111111114</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="13">
+      <c r="A13" s="12">
         <v>12</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="13" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="3">
@@ -1602,31 +1376,35 @@
       <c r="F13" s="3">
         <v>175.3</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="2">
+        <f t="shared" si="2"/>
         <v>678.6</v>
       </c>
       <c r="H13">
-        <f>G13/COUNTIF(C13:F13,"&lt;&gt;0")</f>
+        <f t="shared" si="3"/>
+        <v>169.65</v>
       </c>
       <c r="I13">
-        <f>H13/6</f>
+        <f t="shared" si="0"/>
+        <v>28.275000000000002</v>
       </c>
       <c r="J13">
-        <f>I13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.4250000000000007</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="13">
+      <c r="A14" s="12">
         <v>13</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="3">
         <v>166.5</v>
       </c>
-      <c r="D14" s="3">
-        <v>0</v>
+      <c r="D14" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="E14" s="3">
         <v>170.5</v>
@@ -1634,17 +1412,21 @@
       <c r="F14" s="3">
         <v>176.5</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="2">
+        <f t="shared" si="2"/>
         <v>513.5</v>
       </c>
       <c r="H14">
-        <f>G14/COUNTIF(C14:F14,"&lt;&gt;0")</f>
+        <f>G14/3</f>
+        <v>171.16666666666666</v>
       </c>
       <c r="I14">
-        <f>H14/6</f>
+        <f t="shared" si="0"/>
+        <v>28.527777777777775</v>
       </c>
       <c r="J14">
-        <f>I14/3</f>
+        <f t="shared" si="1"/>
+        <v>9.5092592592592577</v>
       </c>
     </row>
   </sheetData>
@@ -1653,433 +1435,446 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="33.5" style="9" customWidth="1"/>
-    <col min="3" max="4" width="12.6640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" style="9" customWidth="1"/>
-    <col min="6" max="7" width="12.6640625" style="9" customWidth="1"/>
-    <col min="8" max="8" width="9.33203125" style="9"/>
-    <col min="9" max="9" width="14.1640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.33203125" style="9"/>
+    <col min="1" max="1" width="3.33203125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="33.5" style="8" customWidth="1"/>
+    <col min="3" max="4" width="12.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" style="8" customWidth="1"/>
+    <col min="6" max="7" width="12.6640625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" style="8"/>
+    <col min="9" max="9" width="14.1640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.33203125" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20"/>
-      <c r="B1" s="21"/>
-      <c r="C1" s="15" t="s">
+      <c r="A1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="I1" s="18" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17">
+      <c r="A2" s="16">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="22">
-        <v>30</v>
-      </c>
-      <c r="D2" s="22">
+      <c r="C2" s="19">
+        <v>30</v>
+      </c>
+      <c r="D2" s="19">
         <v>29.5</v>
       </c>
-      <c r="E2" s="22">
+      <c r="E2" s="19">
         <v>29.8</v>
       </c>
-      <c r="F2" s="22">
+      <c r="F2" s="19">
         <v>29.8</v>
       </c>
-      <c r="G2" s="23">
+      <c r="G2" s="20">
         <v>119.1</v>
       </c>
       <c r="H2">
         <f>G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <v>29.774999999999999</v>
       </c>
       <c r="I2">
-        <f>H2/3</f>
+        <f t="shared" ref="I2:I14" si="0">H2/3</f>
+        <v>9.9249999999999989</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="13">
+      <c r="A3" s="12">
         <v>2</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="26">
+      <c r="C3" s="21">
         <v>29.8</v>
       </c>
-      <c r="D3" s="26">
+      <c r="D3" s="21">
         <v>29.3</v>
       </c>
-      <c r="E3" s="26">
+      <c r="E3" s="21">
         <v>29.6</v>
       </c>
-      <c r="F3" s="26">
+      <c r="F3" s="21">
         <v>29.5</v>
       </c>
-      <c r="G3" s="27">
+      <c r="G3" s="22">
         <v>118.2</v>
       </c>
       <c r="H3">
-        <f>G3/COUNTIF(C3:F3,"&lt;&gt;0")</f>
+        <f t="shared" ref="H3:H14" si="1">G3/COUNTIF(C3:F3,"&lt;&gt;0")</f>
+        <v>29.55</v>
       </c>
       <c r="I3">
-        <f>H3/3</f>
+        <f t="shared" si="0"/>
+        <v>9.85</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="13">
+      <c r="A4" s="12">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="26">
+      <c r="C4" s="21">
         <v>29.9</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="21">
         <v>28.9</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="21">
         <v>29.3</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="21">
         <v>29.7</v>
       </c>
-      <c r="G4" s="27">
+      <c r="G4" s="22">
         <v>117.8</v>
       </c>
       <c r="H4">
-        <f>G4/COUNTIF(C4:F4,"&lt;&gt;0")</f>
+        <f t="shared" si="1"/>
+        <v>29.45</v>
       </c>
       <c r="I4">
-        <f>H4/3</f>
+        <f t="shared" si="0"/>
+        <v>9.8166666666666664</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="13">
+      <c r="A5" s="12">
         <v>4</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="21">
         <v>29.7</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="21">
         <v>29.2</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="21">
         <v>28.4</v>
       </c>
-      <c r="F5" s="26">
+      <c r="F5" s="21">
         <v>29.6</v>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="22">
         <v>116.9</v>
       </c>
       <c r="H5">
-        <f>G5/COUNTIF(C5:F5,"&lt;&gt;0")</f>
+        <f t="shared" si="1"/>
+        <v>29.225000000000001</v>
       </c>
       <c r="I5">
-        <f>H5/3</f>
+        <f t="shared" si="0"/>
+        <v>9.7416666666666671</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="13">
+      <c r="A6" s="12">
         <v>5</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="21">
         <v>29.4</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="21">
         <v>28.7</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="21">
         <v>29.4</v>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="21">
         <v>29.4</v>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="22">
         <v>116.9</v>
       </c>
       <c r="H6">
-        <f>G6/COUNTIF(C6:F6,"&lt;&gt;0")</f>
+        <f t="shared" si="1"/>
+        <v>29.225000000000001</v>
       </c>
       <c r="I6">
-        <f>H6/3</f>
+        <f t="shared" si="0"/>
+        <v>9.7416666666666671</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="13">
+      <c r="A7" s="12">
         <v>6</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="21">
         <v>28.7</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="21">
         <v>28.5</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="21">
         <v>29.2</v>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="21">
         <v>29.8</v>
       </c>
-      <c r="G7" s="27">
+      <c r="G7" s="22">
         <v>116.2</v>
       </c>
       <c r="H7">
-        <f>G7/COUNTIF(C7:F7,"&lt;&gt;0")</f>
+        <f t="shared" si="1"/>
+        <v>29.05</v>
       </c>
       <c r="I7">
-        <f>H7/3</f>
+        <f t="shared" si="0"/>
+        <v>9.6833333333333336</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="13">
+      <c r="A8" s="12">
         <v>7</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="21">
         <v>28.2</v>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="21">
         <v>29.1</v>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="21">
         <v>29.2</v>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="21">
         <v>29.2</v>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="22">
         <v>115.7</v>
       </c>
       <c r="H8">
-        <f>G8/COUNTIF(C8:F8,"&lt;&gt;0")</f>
+        <f t="shared" si="1"/>
+        <v>28.925000000000001</v>
       </c>
       <c r="I8">
-        <f>H8/3</f>
+        <f t="shared" si="0"/>
+        <v>9.6416666666666675</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="13">
+      <c r="A9" s="12">
         <v>8</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="21">
         <v>28.7</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="21">
         <v>28.1</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="21">
         <v>28.5</v>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="21">
         <v>29.6</v>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="22">
         <v>114.9</v>
       </c>
       <c r="H9">
-        <f>G9/COUNTIF(C9:F9,"&lt;&gt;0")</f>
+        <f t="shared" si="1"/>
+        <v>28.725000000000001</v>
       </c>
       <c r="I9">
-        <f>H9/3</f>
+        <f t="shared" si="0"/>
+        <v>9.5750000000000011</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="13">
+      <c r="A10" s="12">
         <v>9</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="21">
         <v>29.1</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="21">
         <v>28</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="21">
         <v>27.7</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="21">
         <v>29.5</v>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="22">
         <v>114.3</v>
       </c>
       <c r="H10">
-        <f>G10/COUNTIF(C10:F10,"&lt;&gt;0")</f>
+        <f t="shared" si="1"/>
+        <v>28.574999999999999</v>
       </c>
       <c r="I10">
-        <f>H10/3</f>
+        <f t="shared" si="0"/>
+        <v>9.5250000000000004</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="13">
+      <c r="A11" s="12">
         <v>10</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="21">
         <v>27.5</v>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="21">
         <v>28.8</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="21">
         <v>28.1</v>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="21">
         <v>29.4</v>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="22">
         <v>113.8</v>
       </c>
       <c r="H11">
-        <f>G11/COUNTIF(C11:F11,"&lt;&gt;0")</f>
+        <f t="shared" si="1"/>
+        <v>28.45</v>
       </c>
       <c r="I11">
-        <f>H11/3</f>
+        <f t="shared" si="0"/>
+        <v>9.4833333333333325</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="13">
+      <c r="A12" s="12">
         <v>11</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="21">
         <v>28.3</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="21">
         <v>27.6</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="21">
         <v>27</v>
       </c>
-      <c r="F12" s="26">
+      <c r="F12" s="21">
         <v>28.9</v>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="22">
         <v>111.8</v>
       </c>
       <c r="H12">
-        <f>G12/COUNTIF(C12:F12,"&lt;&gt;0")</f>
+        <f t="shared" si="1"/>
+        <v>27.95</v>
       </c>
       <c r="I12">
-        <f>H12/3</f>
+        <f t="shared" si="0"/>
+        <v>9.3166666666666664</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13">
+      <c r="A13" s="12">
         <v>12</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="21">
         <v>26.9</v>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="21">
         <v>27.3</v>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="21">
         <v>26.3</v>
       </c>
-      <c r="F13" s="26">
+      <c r="F13" s="21">
         <v>28.7</v>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="22">
         <v>109.2</v>
       </c>
       <c r="H13">
-        <f>G13/COUNTIF(C13:F13,"&lt;&gt;0")</f>
+        <f t="shared" si="1"/>
+        <v>27.3</v>
       </c>
       <c r="I13">
-        <f>H13/3</f>
+        <f t="shared" si="0"/>
+        <v>9.1</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13">
+      <c r="A14" s="12">
         <v>13</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="21">
         <v>28</v>
       </c>
-      <c r="D14" s="26">
-        <v>0</v>
-      </c>
-      <c r="E14" s="26">
+      <c r="D14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="21">
         <v>26.8</v>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="21">
         <v>29.1</v>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="22">
         <v>83.9</v>
       </c>
       <c r="H14">
-        <f>G14/COUNTIF(C14:F14,"&lt;&gt;0")</f>
+        <f>G14/3</f>
+        <v>27.966666666666669</v>
       </c>
       <c r="I14">
-        <f>H14/3</f>
-      </c>
-    </row>
-    <row r="17" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="18" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="19" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="20" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="21" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="22" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="23" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="24" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="25" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="26" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="27" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="28" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="29" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
+        <f t="shared" si="0"/>
+        <v>9.3222222222222229</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
@@ -2088,433 +1883,446 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="33.5" style="9" customWidth="1"/>
-    <col min="3" max="4" width="12.6640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" style="9" customWidth="1"/>
-    <col min="6" max="7" width="12.6640625" style="9" customWidth="1"/>
-    <col min="8" max="8" width="9.33203125" style="9"/>
-    <col min="9" max="9" width="14.1640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.33203125" style="9"/>
+    <col min="1" max="1" width="3.33203125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="33.5" style="8" customWidth="1"/>
+    <col min="3" max="4" width="12.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" style="8" customWidth="1"/>
+    <col min="6" max="7" width="12.6640625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" style="8"/>
+    <col min="9" max="9" width="14.1640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.33203125" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20"/>
-      <c r="B1" s="21"/>
-      <c r="C1" s="15" t="s">
+      <c r="A1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="I1" s="18" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17">
+      <c r="A2" s="16">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="22">
-        <v>30</v>
-      </c>
-      <c r="D2" s="22">
+      <c r="C2" s="19">
+        <v>30</v>
+      </c>
+      <c r="D2" s="19">
         <v>29.8</v>
       </c>
-      <c r="E2" s="22">
-        <v>30</v>
-      </c>
-      <c r="F2" s="22">
-        <v>30</v>
-      </c>
-      <c r="G2" s="23">
+      <c r="E2" s="19">
+        <v>30</v>
+      </c>
+      <c r="F2" s="19">
+        <v>30</v>
+      </c>
+      <c r="G2" s="20">
         <v>119.8</v>
       </c>
       <c r="H2">
-        <f>G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <f t="shared" ref="H2:H14" si="0">G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <v>29.95</v>
       </c>
       <c r="I2">
-        <f>H2/3</f>
+        <f t="shared" ref="I2:I14" si="1">H2/3</f>
+        <v>9.9833333333333325</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="13">
+      <c r="A3" s="12">
         <v>2</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="26">
+      <c r="C3" s="21">
         <v>29.7</v>
       </c>
-      <c r="D3" s="26">
+      <c r="D3" s="21">
         <v>29.8</v>
       </c>
-      <c r="E3" s="26">
-        <v>30</v>
-      </c>
-      <c r="F3" s="26">
-        <v>30</v>
-      </c>
-      <c r="G3" s="27">
+      <c r="E3" s="21">
+        <v>30</v>
+      </c>
+      <c r="F3" s="21">
+        <v>30</v>
+      </c>
+      <c r="G3" s="22">
         <v>119.5</v>
       </c>
       <c r="H3">
-        <f>G3/COUNTIF(C3:F3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.875</v>
       </c>
       <c r="I3">
-        <f>H3/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9583333333333339</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="13">
+      <c r="A4" s="12">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="26">
+      <c r="C4" s="21">
         <v>29.9</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="21">
         <v>29.8</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="21">
         <v>29.7</v>
       </c>
-      <c r="F4" s="26">
-        <v>30</v>
-      </c>
-      <c r="G4" s="27">
+      <c r="F4" s="21">
+        <v>30</v>
+      </c>
+      <c r="G4" s="22">
         <v>119.4</v>
       </c>
       <c r="H4">
-        <f>G4/COUNTIF(C4:F4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.85</v>
       </c>
       <c r="I4">
-        <f>H4/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9500000000000011</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="13">
+      <c r="A5" s="12">
         <v>4</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="26">
-        <v>30</v>
-      </c>
-      <c r="D5" s="26">
+      <c r="C5" s="21">
+        <v>30</v>
+      </c>
+      <c r="D5" s="21">
         <v>29.1</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="21">
         <v>29.8</v>
       </c>
-      <c r="F5" s="26">
+      <c r="F5" s="21">
         <v>29.8</v>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="22">
         <v>118.7</v>
       </c>
       <c r="H5">
-        <f>G5/COUNTIF(C5:F5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.675000000000001</v>
       </c>
       <c r="I5">
-        <f>H5/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8916666666666675</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="13">
+      <c r="A6" s="12">
         <v>5</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="21">
         <v>29.9</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="21">
         <v>29.6</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="21">
         <v>28.5</v>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="21">
         <v>29.9</v>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="22">
         <v>117.9</v>
       </c>
       <c r="H6">
-        <f>G6/COUNTIF(C6:F6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.475000000000001</v>
       </c>
       <c r="I6">
-        <f>H6/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8250000000000011</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="13">
+      <c r="A7" s="12">
         <v>6</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="26">
-        <v>30</v>
-      </c>
-      <c r="D7" s="26">
+      <c r="C7" s="21">
+        <v>30</v>
+      </c>
+      <c r="D7" s="21">
         <v>29.1</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="21">
         <v>28.8</v>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="21">
         <v>29.9</v>
       </c>
-      <c r="G7" s="27">
+      <c r="G7" s="22">
         <v>117.8</v>
       </c>
       <c r="H7">
-        <f>G7/COUNTIF(C7:F7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.45</v>
       </c>
       <c r="I7">
-        <f>H7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8166666666666664</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="13">
+      <c r="A8" s="12">
         <v>7</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="21">
         <v>29.5</v>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="21">
         <v>28.4</v>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="21">
         <v>29.7</v>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="21">
         <v>29.8</v>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="22">
         <v>117.4</v>
       </c>
       <c r="H8">
-        <f>G8/COUNTIF(C8:F8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.35</v>
       </c>
       <c r="I8">
-        <f>H8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7833333333333332</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="13">
+      <c r="A9" s="12">
         <v>8</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="21">
         <v>28.9</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="21">
         <v>29</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="21">
         <v>29.5</v>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="21">
         <v>29.7</v>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="22">
         <v>117.1</v>
       </c>
       <c r="H9">
-        <f>G9/COUNTIF(C9:F9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.274999999999999</v>
       </c>
       <c r="I9">
-        <f>H9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7583333333333329</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="13">
+      <c r="A10" s="12">
         <v>9</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="21">
         <v>28.9</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="21">
         <v>28.8</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="21">
         <v>29</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="21">
         <v>29.9</v>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="22">
         <v>116.6</v>
       </c>
       <c r="H10">
-        <f>G10/COUNTIF(C10:F10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.15</v>
       </c>
       <c r="I10">
-        <f>H10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7166666666666668</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="13">
+      <c r="A11" s="12">
         <v>10</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="21">
         <v>28.3</v>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="21">
         <v>28.8</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="21">
         <v>29.8</v>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="21">
         <v>29.3</v>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="22">
         <v>116.2</v>
       </c>
       <c r="H11">
-        <f>G11/COUNTIF(C11:F11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.05</v>
       </c>
       <c r="I11">
-        <f>H11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6833333333333336</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="13">
+      <c r="A12" s="12">
         <v>11</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="21">
         <v>28.1</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="21">
         <v>28.5</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="21">
         <v>27.5</v>
       </c>
-      <c r="F12" s="26">
+      <c r="F12" s="21">
         <v>29.4</v>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="22">
         <v>113.5</v>
       </c>
       <c r="H12">
-        <f>G12/COUNTIF(C12:F12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.375</v>
       </c>
       <c r="I12">
-        <f>H12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.4583333333333339</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13">
+      <c r="A13" s="12">
         <v>12</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="21">
         <v>28.5</v>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="21">
         <v>28.5</v>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="21">
         <v>26.6</v>
       </c>
-      <c r="F13" s="26">
+      <c r="F13" s="21">
         <v>29.4</v>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="22">
         <v>113</v>
       </c>
       <c r="H13">
-        <f>G13/COUNTIF(C13:F13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.25</v>
       </c>
       <c r="I13">
-        <f>H13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.4166666666666661</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13">
+      <c r="A14" s="12">
         <v>13</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="21">
         <v>27.5</v>
       </c>
-      <c r="D14" s="26">
-        <v>0</v>
-      </c>
-      <c r="E14" s="26">
+      <c r="D14" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="21">
         <v>29</v>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="21">
         <v>29.8</v>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="22">
         <v>86.3</v>
       </c>
       <c r="H14">
-        <f>G14/COUNTIF(C14:F14,"&lt;&gt;0")</f>
+        <f>G14/3</f>
+        <v>28.766666666666666</v>
       </c>
       <c r="I14">
-        <f>H14/3</f>
-      </c>
-    </row>
-    <row r="17" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="18" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="19" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="20" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="21" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="22" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="23" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="24" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="25" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="26" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="27" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="28" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="29" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
+        <f t="shared" si="1"/>
+        <v>9.5888888888888886</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
@@ -2523,421 +2331,447 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="33.5" style="9" customWidth="1"/>
-    <col min="3" max="4" width="12.6640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" style="9" customWidth="1"/>
-    <col min="6" max="7" width="12.6640625" style="9" customWidth="1"/>
-    <col min="8" max="8" width="9.33203125" style="9"/>
-    <col min="9" max="9" width="14.1640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.33203125" style="9"/>
+    <col min="1" max="1" width="3.33203125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="33.5" style="8" customWidth="1"/>
+    <col min="3" max="4" width="12.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" style="8" customWidth="1"/>
+    <col min="6" max="7" width="12.6640625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" style="8"/>
+    <col min="9" max="9" width="14.1640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.33203125" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20"/>
-      <c r="B1" s="21"/>
-      <c r="C1" s="15" t="s">
+      <c r="A1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="I1" s="18" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17">
+      <c r="A2" s="16">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="22">
-        <v>30</v>
-      </c>
-      <c r="D2" s="22">
+      <c r="C2" s="19">
+        <v>30</v>
+      </c>
+      <c r="D2" s="19">
         <v>29.8</v>
       </c>
-      <c r="E2" s="22">
+      <c r="E2" s="19">
         <v>29.8</v>
       </c>
-      <c r="F2" s="22">
+      <c r="F2" s="19">
         <v>29.9</v>
       </c>
-      <c r="G2" s="23">
+      <c r="G2" s="20">
         <v>119.5</v>
       </c>
       <c r="H2">
-        <f>G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <f t="shared" ref="H2:H14" si="0">G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <v>29.875</v>
       </c>
       <c r="I2">
-        <f>H2/3</f>
+        <f t="shared" ref="I2:I14" si="1">H2/3</f>
+        <v>9.9583333333333339</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="13">
+      <c r="A3" s="12">
         <v>2</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="26">
-        <v>30</v>
-      </c>
-      <c r="D3" s="26">
-        <v>30</v>
-      </c>
-      <c r="E3" s="26">
+      <c r="C3" s="21">
+        <v>30</v>
+      </c>
+      <c r="D3" s="21">
+        <v>30</v>
+      </c>
+      <c r="E3" s="21">
         <v>29.5</v>
       </c>
-      <c r="F3" s="26">
+      <c r="F3" s="21">
         <v>29.9</v>
       </c>
-      <c r="G3" s="27">
+      <c r="G3" s="22">
         <v>119.4</v>
       </c>
       <c r="H3">
-        <f>G3/COUNTIF(C3:F3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.85</v>
       </c>
       <c r="I3">
-        <f>H3/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9500000000000011</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="13">
+      <c r="A4" s="12">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="26">
-        <v>30</v>
-      </c>
-      <c r="D4" s="26">
+      <c r="C4" s="21">
+        <v>30</v>
+      </c>
+      <c r="D4" s="21">
         <v>29.6</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="21">
         <v>29.7</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="21">
         <v>29.9</v>
       </c>
-      <c r="G4" s="27">
+      <c r="G4" s="22">
         <v>119.2</v>
       </c>
       <c r="H4">
-        <f>G4/COUNTIF(C4:F4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.8</v>
       </c>
       <c r="I4">
-        <f>H4/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9333333333333336</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="13">
+      <c r="A5" s="12">
         <v>4</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="26">
-        <v>30</v>
-      </c>
-      <c r="D5" s="26">
+      <c r="C5" s="21">
+        <v>30</v>
+      </c>
+      <c r="D5" s="21">
         <v>29.9</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="21">
         <v>29.1</v>
       </c>
-      <c r="F5" s="26">
+      <c r="F5" s="21">
         <v>29.9</v>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="22">
         <v>118.9</v>
       </c>
       <c r="H5">
-        <f>G5/COUNTIF(C5:F5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.725000000000001</v>
       </c>
       <c r="I5">
-        <f>H5/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9083333333333332</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="13">
+      <c r="A6" s="12">
         <v>5</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="26">
-        <v>30</v>
-      </c>
-      <c r="D6" s="26">
+      <c r="C6" s="21">
+        <v>30</v>
+      </c>
+      <c r="D6" s="21">
         <v>29.2</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="21">
         <v>29.8</v>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="21">
         <v>29.9</v>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="22">
         <v>118.9</v>
       </c>
       <c r="H6">
-        <f>G6/COUNTIF(C6:F6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.725000000000001</v>
       </c>
       <c r="I6">
-        <f>H6/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9083333333333332</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="13">
+      <c r="A7" s="12">
         <v>6</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="21">
         <v>29.1</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="21">
         <v>28.9</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="21">
         <v>29.4</v>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="21">
         <v>29.9</v>
       </c>
-      <c r="G7" s="27">
+      <c r="G7" s="22">
         <v>117.3</v>
       </c>
       <c r="H7">
-        <f>G7/COUNTIF(C7:F7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.324999999999999</v>
       </c>
       <c r="I7">
-        <f>H7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7750000000000004</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="13">
+      <c r="A8" s="12">
         <v>7</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="21">
         <v>28.4</v>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="21">
         <v>29.5</v>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="21">
         <v>29.1</v>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="21">
         <v>29.6</v>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="22">
         <v>116.6</v>
       </c>
       <c r="H8">
-        <f>G8/COUNTIF(C8:F8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.15</v>
       </c>
       <c r="I8">
-        <f>H8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7166666666666668</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="13">
+      <c r="A9" s="12">
         <v>8</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="21">
         <v>28.7</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="21">
         <v>28.9</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="21">
         <v>28.4</v>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="21">
         <v>29.7</v>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="22">
         <v>115.7</v>
       </c>
       <c r="H9">
-        <f>G9/COUNTIF(C9:F9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.925000000000001</v>
       </c>
       <c r="I9">
-        <f>H9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6416666666666675</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="13">
+      <c r="A10" s="12">
         <v>9</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="21">
         <v>28.5</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="21">
         <v>28.7</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="21">
         <v>28.9</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="21">
         <v>29.3</v>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="22">
         <v>115.4</v>
       </c>
       <c r="H10">
-        <f>G10/COUNTIF(C10:F10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.85</v>
       </c>
       <c r="I10">
-        <f>H10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6166666666666671</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="13">
+      <c r="A11" s="12">
         <v>10</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="21">
         <v>29.4</v>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="21">
         <v>28.1</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="21">
         <v>28.2</v>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="21">
         <v>29.5</v>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="22">
         <v>115.2</v>
       </c>
       <c r="H11">
-        <f>G11/COUNTIF(C11:F11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.8</v>
       </c>
       <c r="I11">
-        <f>H11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="13">
+      <c r="A12" s="12">
         <v>11</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="21">
         <v>28.7</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="21">
         <v>28.3</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="21">
         <v>27.9</v>
       </c>
-      <c r="F12" s="26">
+      <c r="F12" s="21">
         <v>29.2</v>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="22">
         <v>114.1</v>
       </c>
       <c r="H12">
-        <f>G12/COUNTIF(C12:F12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.524999999999999</v>
       </c>
       <c r="I12">
-        <f>H12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.5083333333333329</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13">
+      <c r="A13" s="12">
         <v>12</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="21">
         <v>27.7</v>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="21">
         <v>27.6</v>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="21">
         <v>27.1</v>
       </c>
-      <c r="F13" s="26">
+      <c r="F13" s="21">
         <v>28.9</v>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="22">
         <v>111.3</v>
       </c>
       <c r="H13">
-        <f>G13/COUNTIF(C13:F13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>27.824999999999999</v>
       </c>
       <c r="I13">
-        <f>H13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.2750000000000004</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13">
+      <c r="A14" s="12">
         <v>13</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="21">
         <v>27.3</v>
       </c>
-      <c r="D14" s="26">
-        <v>0</v>
-      </c>
-      <c r="E14" s="26">
+      <c r="D14" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="21">
         <v>27.6</v>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="21">
         <v>29.3</v>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="22">
         <v>84.2</v>
       </c>
       <c r="H14">
-        <f>G14/COUNTIF(C14:F14,"&lt;&gt;0")</f>
+        <f>G14/3</f>
+        <v>28.066666666666666</v>
       </c>
       <c r="I14">
-        <f>H14/3</f>
+        <f t="shared" si="1"/>
+        <v>9.3555555555555561</v>
       </c>
     </row>
   </sheetData>
@@ -2948,416 +2782,442 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="33.5" style="9" customWidth="1"/>
-    <col min="3" max="4" width="12.6640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" style="9" customWidth="1"/>
-    <col min="6" max="7" width="12.6640625" style="9" customWidth="1"/>
-    <col min="8" max="8" width="9.33203125" style="9"/>
-    <col min="9" max="9" width="14.1640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.33203125" style="9"/>
+    <col min="1" max="1" width="3.33203125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="33.5" style="8" customWidth="1"/>
+    <col min="3" max="4" width="12.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" style="8" customWidth="1"/>
+    <col min="6" max="7" width="12.6640625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" style="8"/>
+    <col min="9" max="9" width="14.1640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.33203125" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20"/>
-      <c r="B1" s="21"/>
-      <c r="C1" s="15" t="s">
+      <c r="A1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="I1" s="18" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17">
+      <c r="A2" s="16">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="22">
-        <v>30</v>
-      </c>
-      <c r="D2" s="22">
-        <v>30</v>
-      </c>
-      <c r="E2" s="22">
-        <v>30</v>
-      </c>
-      <c r="F2" s="22">
+      <c r="C2" s="19">
+        <v>30</v>
+      </c>
+      <c r="D2" s="19">
+        <v>30</v>
+      </c>
+      <c r="E2" s="19">
+        <v>30</v>
+      </c>
+      <c r="F2" s="19">
         <v>29.9</v>
       </c>
-      <c r="G2" s="23">
+      <c r="G2" s="20">
         <v>119.9</v>
       </c>
       <c r="H2">
-        <f>G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <f t="shared" ref="H2:H14" si="0">G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <v>29.975000000000001</v>
       </c>
       <c r="I2">
-        <f>H2/3</f>
+        <f t="shared" ref="I2:I14" si="1">H2/3</f>
+        <v>9.9916666666666671</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="13"/>
-      <c r="B3" s="14" t="s">
+      <c r="A3" s="12"/>
+      <c r="B3" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="26">
-        <v>30</v>
-      </c>
-      <c r="D3" s="26">
+      <c r="C3" s="21">
+        <v>30</v>
+      </c>
+      <c r="D3" s="21">
         <v>29.9</v>
       </c>
-      <c r="E3" s="26">
-        <v>30</v>
-      </c>
-      <c r="F3" s="26">
-        <v>30</v>
-      </c>
-      <c r="G3" s="27">
+      <c r="E3" s="21">
+        <v>30</v>
+      </c>
+      <c r="F3" s="21">
+        <v>30</v>
+      </c>
+      <c r="G3" s="22">
         <v>119.9</v>
       </c>
       <c r="H3">
-        <f>G3/COUNTIF(C3:F3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.975000000000001</v>
       </c>
       <c r="I3">
-        <f>H3/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9916666666666671</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="13">
+      <c r="A4" s="12">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="26">
-        <v>30</v>
-      </c>
-      <c r="D4" s="26">
+      <c r="C4" s="21">
+        <v>30</v>
+      </c>
+      <c r="D4" s="21">
         <v>29.8</v>
       </c>
-      <c r="E4" s="26">
-        <v>30</v>
-      </c>
-      <c r="F4" s="26">
-        <v>30</v>
-      </c>
-      <c r="G4" s="27">
+      <c r="E4" s="21">
+        <v>30</v>
+      </c>
+      <c r="F4" s="21">
+        <v>30</v>
+      </c>
+      <c r="G4" s="22">
         <v>119.8</v>
       </c>
       <c r="H4">
-        <f>G4/COUNTIF(C4:F4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.95</v>
       </c>
       <c r="I4">
-        <f>H4/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9833333333333325</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="13">
+      <c r="A5" s="12">
         <v>4</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="21">
         <v>29.9</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="21">
         <v>29.8</v>
       </c>
-      <c r="E5" s="26">
-        <v>30</v>
-      </c>
-      <c r="F5" s="26">
+      <c r="E5" s="21">
+        <v>30</v>
+      </c>
+      <c r="F5" s="21">
         <v>29.7</v>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="22">
         <v>119.4</v>
       </c>
       <c r="H5">
-        <f>G5/COUNTIF(C5:F5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.85</v>
       </c>
       <c r="I5">
-        <f>H5/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9500000000000011</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="13">
+      <c r="A6" s="12">
         <v>5</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="26">
-        <v>30</v>
-      </c>
-      <c r="D6" s="26">
+      <c r="C6" s="21">
+        <v>30</v>
+      </c>
+      <c r="D6" s="21">
         <v>29.7</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="21">
         <v>29.8</v>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="21">
         <v>29.7</v>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="22">
         <v>119.2</v>
       </c>
       <c r="H6">
-        <f>G6/COUNTIF(C6:F6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.8</v>
       </c>
       <c r="I6">
-        <f>H6/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9333333333333336</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="13">
+      <c r="A7" s="12">
         <v>6</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="21">
         <v>29.5</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="21">
         <v>29.6</v>
       </c>
-      <c r="E7" s="26">
-        <v>30</v>
-      </c>
-      <c r="F7" s="26">
+      <c r="E7" s="21">
+        <v>30</v>
+      </c>
+      <c r="F7" s="21">
         <v>29.9</v>
       </c>
-      <c r="G7" s="27">
+      <c r="G7" s="22">
         <v>119</v>
       </c>
       <c r="H7">
-        <f>G7/COUNTIF(C7:F7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.75</v>
       </c>
       <c r="I7">
-        <f>H7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9166666666666661</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="13">
+      <c r="A8" s="12">
         <v>7</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="26">
-        <v>30</v>
-      </c>
-      <c r="D8" s="26">
+      <c r="C8" s="21">
+        <v>30</v>
+      </c>
+      <c r="D8" s="21">
         <v>29.1</v>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="21">
         <v>29.9</v>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="21">
         <v>29.9</v>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="22">
         <v>118.9</v>
       </c>
       <c r="H8">
-        <f>G8/COUNTIF(C8:F8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.725000000000001</v>
       </c>
       <c r="I8">
-        <f>H8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9083333333333332</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="13">
+      <c r="A9" s="12">
         <v>8</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="21">
         <v>29.7</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="21">
         <v>29.5</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="21">
         <v>29.8</v>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="21">
         <v>29.7</v>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="22">
         <v>118.7</v>
       </c>
       <c r="H9">
-        <f>G9/COUNTIF(C9:F9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.675000000000001</v>
       </c>
       <c r="I9">
-        <f>H9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8916666666666675</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="13">
+      <c r="A10" s="12">
         <v>9</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="21">
         <v>28.6</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="21">
         <v>29.1</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="21">
         <v>29.7</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="21">
         <v>29.5</v>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="22">
         <v>116.9</v>
       </c>
       <c r="H10">
-        <f>G10/COUNTIF(C10:F10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.225000000000001</v>
       </c>
       <c r="I10">
-        <f>H10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7416666666666671</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="13">
+      <c r="A11" s="12">
         <v>10</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="21">
         <v>28.3</v>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="21">
         <v>29.4</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="21">
         <v>29.2</v>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="21">
         <v>29.7</v>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="22">
         <v>116.6</v>
       </c>
       <c r="H11">
-        <f>G11/COUNTIF(C11:F11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.15</v>
       </c>
       <c r="I11">
-        <f>H11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7166666666666668</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="13">
+      <c r="A12" s="12">
         <v>11</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="21">
         <v>28.8</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="21">
         <v>29.3</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="21">
         <v>28.3</v>
       </c>
-      <c r="F12" s="26">
+      <c r="F12" s="21">
         <v>29.6</v>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="22">
         <v>116</v>
       </c>
       <c r="H12">
-        <f>G12/COUNTIF(C12:F12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29</v>
       </c>
       <c r="I12">
-        <f>H12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6666666666666661</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13">
+      <c r="A13" s="12">
         <v>12</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="21">
         <v>27.8</v>
       </c>
-      <c r="D13" s="26">
-        <v>30</v>
-      </c>
-      <c r="E13" s="26">
+      <c r="D13" s="21">
+        <v>30</v>
+      </c>
+      <c r="E13" s="21">
         <v>28.2</v>
       </c>
-      <c r="F13" s="26">
+      <c r="F13" s="21">
         <v>29.4</v>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="22">
         <v>115.4</v>
       </c>
       <c r="H13">
-        <f>G13/COUNTIF(C13:F13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.85</v>
       </c>
       <c r="I13">
-        <f>H13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6166666666666671</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13">
+      <c r="A14" s="12">
         <v>13</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="21">
         <v>29.2</v>
       </c>
-      <c r="D14" s="26">
-        <v>0</v>
-      </c>
-      <c r="E14" s="26">
+      <c r="D14" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="21">
         <v>29.8</v>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="21">
         <v>29.2</v>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="22">
         <v>88.2</v>
       </c>
       <c r="H14">
-        <f>G14/COUNTIF(C14:F14,"&lt;&gt;0")</f>
+        <f>G14/3</f>
+        <v>29.400000000000002</v>
       </c>
       <c r="I14">
-        <f>H14/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8000000000000007</v>
       </c>
     </row>
   </sheetData>
@@ -3368,418 +3228,444 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="33.5" style="9" customWidth="1"/>
-    <col min="3" max="4" width="12.6640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" style="9" customWidth="1"/>
-    <col min="6" max="7" width="12.6640625" style="9" customWidth="1"/>
-    <col min="8" max="8" width="9.33203125" style="9"/>
-    <col min="9" max="9" width="14.1640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.33203125" style="9"/>
+    <col min="1" max="1" width="3.33203125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="33.5" style="8" customWidth="1"/>
+    <col min="3" max="4" width="12.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" style="8" customWidth="1"/>
+    <col min="6" max="7" width="12.6640625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" style="8"/>
+    <col min="9" max="9" width="14.1640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.33203125" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20"/>
-      <c r="B1" s="21"/>
-      <c r="C1" s="15" t="s">
+      <c r="A1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="I1" s="18" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17">
+      <c r="A2" s="16">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="22">
-        <v>30</v>
-      </c>
-      <c r="D2" s="22">
+      <c r="C2" s="19">
+        <v>30</v>
+      </c>
+      <c r="D2" s="19">
         <v>29.9</v>
       </c>
-      <c r="E2" s="22">
-        <v>30</v>
-      </c>
-      <c r="F2" s="22">
-        <v>30</v>
-      </c>
-      <c r="G2" s="23">
+      <c r="E2" s="19">
+        <v>30</v>
+      </c>
+      <c r="F2" s="19">
+        <v>30</v>
+      </c>
+      <c r="G2" s="20">
         <v>119.9</v>
       </c>
       <c r="H2">
-        <f>G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <f t="shared" ref="H2:H14" si="0">G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <v>29.975000000000001</v>
       </c>
       <c r="I2">
-        <f>H2/3</f>
+        <f t="shared" ref="I2:I14" si="1">H2/3</f>
+        <v>9.9916666666666671</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="13">
+      <c r="A3" s="12">
         <v>2</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="26">
-        <v>30</v>
-      </c>
-      <c r="D3" s="26">
+      <c r="C3" s="21">
+        <v>30</v>
+      </c>
+      <c r="D3" s="21">
         <v>29.8</v>
       </c>
-      <c r="E3" s="26">
+      <c r="E3" s="21">
         <v>29.9</v>
       </c>
-      <c r="F3" s="26">
-        <v>30</v>
-      </c>
-      <c r="G3" s="27">
+      <c r="F3" s="21">
+        <v>30</v>
+      </c>
+      <c r="G3" s="22">
         <v>119.7</v>
       </c>
       <c r="H3">
-        <f>G3/COUNTIF(C3:F3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.925000000000001</v>
       </c>
       <c r="I3">
-        <f>H3/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9749999999999996</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="13">
+      <c r="A4" s="12">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="26">
+      <c r="C4" s="21">
         <v>29.8</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="21">
         <v>29.6</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="21">
         <v>29.6</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="21">
         <v>29.8</v>
       </c>
-      <c r="G4" s="27">
+      <c r="G4" s="22">
         <v>118.8</v>
       </c>
       <c r="H4">
-        <f>G4/COUNTIF(C4:F4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.7</v>
       </c>
       <c r="I4">
-        <f>H4/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="13">
+      <c r="A5" s="12">
         <v>4</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="26">
-        <v>30</v>
-      </c>
-      <c r="D5" s="26">
+      <c r="C5" s="21">
+        <v>30</v>
+      </c>
+      <c r="D5" s="21">
         <v>29.1</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="21">
         <v>29.8</v>
       </c>
-      <c r="F5" s="26">
+      <c r="F5" s="21">
         <v>29.6</v>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="22">
         <v>118.5</v>
       </c>
       <c r="H5">
-        <f>G5/COUNTIF(C5:F5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.625</v>
       </c>
       <c r="I5">
-        <f>H5/3</f>
+        <f t="shared" si="1"/>
+        <v>9.875</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="13">
+      <c r="A6" s="12">
         <v>5</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="21">
         <v>29.6</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="21">
         <v>29.2</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="21">
         <v>29.7</v>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="21">
         <v>29.9</v>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="22">
         <v>118.4</v>
       </c>
       <c r="H6">
-        <f>G6/COUNTIF(C6:F6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.6</v>
       </c>
       <c r="I6">
-        <f>H6/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8666666666666671</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="13">
+      <c r="A7" s="12">
         <v>6</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="21">
         <v>29.5</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="21">
         <v>29.7</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="21">
         <v>29</v>
       </c>
-      <c r="F7" s="26">
-        <v>30</v>
-      </c>
-      <c r="G7" s="27">
+      <c r="F7" s="21">
+        <v>30</v>
+      </c>
+      <c r="G7" s="22">
         <v>118.2</v>
       </c>
       <c r="H7">
-        <f>G7/COUNTIF(C7:F7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.55</v>
       </c>
       <c r="I7">
-        <f>H7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.85</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="13">
+      <c r="A8" s="12">
         <v>7</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="21">
         <v>28.7</v>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="21">
         <v>29</v>
       </c>
-      <c r="E8" s="26">
-        <v>30</v>
-      </c>
-      <c r="F8" s="26">
+      <c r="E8" s="21">
+        <v>30</v>
+      </c>
+      <c r="F8" s="21">
         <v>29.9</v>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="22">
         <v>117.6</v>
       </c>
       <c r="H8">
-        <f>G8/COUNTIF(C8:F8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.4</v>
       </c>
       <c r="I8">
-        <f>H8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7999999999999989</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="13">
+      <c r="A9" s="12">
         <v>8</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="21">
         <v>28.4</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="21">
         <v>29.5</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="21">
         <v>29.6</v>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="21">
         <v>29.5</v>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="22">
         <v>117</v>
       </c>
       <c r="H9">
-        <f>G9/COUNTIF(C9:F9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.25</v>
       </c>
       <c r="I9">
-        <f>H9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.75</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="13">
+      <c r="A10" s="12">
         <v>9</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="21">
         <v>28.7</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="21">
         <v>28.7</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="21">
         <v>28.7</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="21">
         <v>29.6</v>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="22">
         <v>115.7</v>
       </c>
       <c r="H10">
-        <f>G10/COUNTIF(C10:F10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.925000000000001</v>
       </c>
       <c r="I10">
-        <f>H10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.6416666666666675</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="13">
+      <c r="A11" s="12">
         <v>10</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="21">
         <v>29.3</v>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="21">
         <v>27.9</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="21">
         <v>28.2</v>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="21">
         <v>29.6</v>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="22">
         <v>115</v>
       </c>
       <c r="H11">
-        <f>G11/COUNTIF(C11:F11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.75</v>
       </c>
       <c r="I11">
-        <f>H11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.5833333333333339</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="13">
+      <c r="A12" s="12">
         <v>11</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="21">
         <v>27.6</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="21">
         <v>28.8</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="21">
         <v>29.1</v>
       </c>
-      <c r="F12" s="26">
+      <c r="F12" s="21">
         <v>29.5</v>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="22">
         <v>115</v>
       </c>
       <c r="H12">
-        <f>G12/COUNTIF(C12:F12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.75</v>
       </c>
       <c r="I12">
-        <f>H12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.5833333333333339</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13">
+      <c r="A13" s="12">
         <v>12</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="21">
         <v>28.9</v>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="21">
         <v>28.9</v>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="21">
         <v>27.6</v>
       </c>
-      <c r="F13" s="26">
+      <c r="F13" s="21">
         <v>29.5</v>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="22">
         <v>114.9</v>
       </c>
       <c r="H13">
-        <f>G13/COUNTIF(C13:F13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>28.725000000000001</v>
       </c>
       <c r="I13">
-        <f>H13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.5750000000000011</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13">
+      <c r="A14" s="12">
         <v>13</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="21">
         <v>27.5</v>
       </c>
-      <c r="D14" s="26">
-        <v>0</v>
-      </c>
-      <c r="E14" s="26">
+      <c r="D14" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="21">
         <v>28.2</v>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="21">
         <v>29.5</v>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="22">
         <v>85.2</v>
       </c>
       <c r="H14">
-        <f>G14/COUNTIF(C14:F14,"&lt;&gt;0")</f>
+        <f>G14/3</f>
+        <v>28.400000000000002</v>
       </c>
       <c r="I14">
-        <f>H14/3</f>
+        <f t="shared" si="1"/>
+        <v>9.4666666666666668</v>
       </c>
     </row>
   </sheetData>
@@ -3790,418 +3676,444 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="33.5" style="9" customWidth="1"/>
-    <col min="3" max="4" width="12.6640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" style="9" customWidth="1"/>
-    <col min="6" max="7" width="12.6640625" style="9" customWidth="1"/>
-    <col min="8" max="8" width="9.33203125" style="9"/>
-    <col min="9" max="9" width="14.1640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.33203125" style="9"/>
+    <col min="1" max="1" width="3.33203125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="33.5" style="8" customWidth="1"/>
+    <col min="3" max="4" width="12.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" style="8" customWidth="1"/>
+    <col min="6" max="7" width="12.6640625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" style="8"/>
+    <col min="9" max="9" width="14.1640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.33203125" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20"/>
-      <c r="B1" s="21"/>
-      <c r="C1" s="15" t="s">
+      <c r="A1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="I1" s="18" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17">
+      <c r="A2" s="16">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="22">
-        <v>30</v>
-      </c>
-      <c r="D2" s="22">
-        <v>30</v>
-      </c>
-      <c r="E2" s="22">
-        <v>30</v>
-      </c>
-      <c r="F2" s="22">
-        <v>30</v>
-      </c>
-      <c r="G2" s="23">
+      <c r="C2" s="19">
+        <v>30</v>
+      </c>
+      <c r="D2" s="19">
+        <v>30</v>
+      </c>
+      <c r="E2" s="19">
+        <v>30</v>
+      </c>
+      <c r="F2" s="19">
+        <v>30</v>
+      </c>
+      <c r="G2" s="20">
         <v>120</v>
       </c>
       <c r="H2">
-        <f>G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <f t="shared" ref="H2:H14" si="0">G2/COUNTIF(C2:F2,"&lt;&gt;0")</f>
+        <v>30</v>
       </c>
       <c r="I2">
-        <f>H2/3</f>
+        <f t="shared" ref="I2:I14" si="1">H2/3</f>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="13">
+      <c r="A3" s="12">
         <v>2</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="26">
-        <v>30</v>
-      </c>
-      <c r="D3" s="26">
-        <v>30</v>
-      </c>
-      <c r="E3" s="26">
+      <c r="C3" s="21">
+        <v>30</v>
+      </c>
+      <c r="D3" s="21">
+        <v>30</v>
+      </c>
+      <c r="E3" s="21">
         <v>29.9</v>
       </c>
-      <c r="F3" s="26">
-        <v>30</v>
-      </c>
-      <c r="G3" s="27">
+      <c r="F3" s="21">
+        <v>30</v>
+      </c>
+      <c r="G3" s="22">
         <v>119.9</v>
       </c>
       <c r="H3">
-        <f>G3/COUNTIF(C3:F3,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.975000000000001</v>
       </c>
       <c r="I3">
-        <f>H3/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9916666666666671</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="13">
+      <c r="A4" s="12">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="26">
-        <v>30</v>
-      </c>
-      <c r="D4" s="26">
+      <c r="C4" s="21">
+        <v>30</v>
+      </c>
+      <c r="D4" s="21">
         <v>29.9</v>
       </c>
-      <c r="E4" s="26">
-        <v>30</v>
-      </c>
-      <c r="F4" s="26">
+      <c r="E4" s="21">
+        <v>30</v>
+      </c>
+      <c r="F4" s="21">
         <v>29.9</v>
       </c>
-      <c r="G4" s="27">
+      <c r="G4" s="22">
         <v>119.8</v>
       </c>
       <c r="H4">
-        <f>G4/COUNTIF(C4:F4,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.95</v>
       </c>
       <c r="I4">
-        <f>H4/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9833333333333325</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="13">
+      <c r="A5" s="12">
         <v>4</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="26">
-        <v>30</v>
-      </c>
-      <c r="D5" s="26">
-        <v>30</v>
-      </c>
-      <c r="E5" s="26">
-        <v>30</v>
-      </c>
-      <c r="F5" s="26">
+      <c r="C5" s="21">
+        <v>30</v>
+      </c>
+      <c r="D5" s="21">
+        <v>30</v>
+      </c>
+      <c r="E5" s="21">
+        <v>30</v>
+      </c>
+      <c r="F5" s="21">
         <v>29.8</v>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="22">
         <v>119.8</v>
       </c>
       <c r="H5">
-        <f>G5/COUNTIF(C5:F5,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.95</v>
       </c>
       <c r="I5">
-        <f>H5/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9833333333333325</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="13">
+      <c r="A6" s="12">
         <v>5</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="26">
-        <v>30</v>
-      </c>
-      <c r="D6" s="26">
+      <c r="C6" s="21">
+        <v>30</v>
+      </c>
+      <c r="D6" s="21">
         <v>29.9</v>
       </c>
-      <c r="E6" s="26">
-        <v>30</v>
-      </c>
-      <c r="F6" s="26">
+      <c r="E6" s="21">
+        <v>30</v>
+      </c>
+      <c r="F6" s="21">
         <v>29.8</v>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="22">
         <v>119.7</v>
       </c>
       <c r="H6">
-        <f>G6/COUNTIF(C6:F6,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.925000000000001</v>
       </c>
       <c r="I6">
-        <f>H6/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9749999999999996</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="13">
+      <c r="A7" s="12">
         <v>6</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="21">
         <v>29.8</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="21">
         <v>29.9</v>
       </c>
-      <c r="E7" s="26">
-        <v>30</v>
-      </c>
-      <c r="F7" s="26">
-        <v>30</v>
-      </c>
-      <c r="G7" s="27">
+      <c r="E7" s="21">
+        <v>30</v>
+      </c>
+      <c r="F7" s="21">
+        <v>30</v>
+      </c>
+      <c r="G7" s="22">
         <v>119.7</v>
       </c>
       <c r="H7">
-        <f>G7/COUNTIF(C7:F7,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.925000000000001</v>
       </c>
       <c r="I7">
-        <f>H7/3</f>
+        <f t="shared" si="1"/>
+        <v>9.9749999999999996</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="13">
+      <c r="A8" s="12">
         <v>7</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="26">
-        <v>30</v>
-      </c>
-      <c r="D8" s="26">
-        <v>30</v>
-      </c>
-      <c r="E8" s="26">
+      <c r="C8" s="21">
+        <v>30</v>
+      </c>
+      <c r="D8" s="21">
+        <v>30</v>
+      </c>
+      <c r="E8" s="21">
         <v>28.8</v>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="21">
         <v>29.8</v>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="22">
         <v>118.6</v>
       </c>
       <c r="H8">
-        <f>G8/COUNTIF(C8:F8,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.65</v>
       </c>
       <c r="I8">
-        <f>H8/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8833333333333329</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="13">
+      <c r="A9" s="12">
         <v>8</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="21">
         <v>29.3</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="21">
         <v>29.8</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="21">
         <v>29.6</v>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="21">
         <v>29.8</v>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="22">
         <v>118.5</v>
       </c>
       <c r="H9">
-        <f>G9/COUNTIF(C9:F9,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.625</v>
       </c>
       <c r="I9">
-        <f>H9/3</f>
+        <f t="shared" si="1"/>
+        <v>9.875</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="13">
+      <c r="A10" s="12">
         <v>9</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="21">
         <v>28.4</v>
       </c>
-      <c r="D10" s="26">
-        <v>30</v>
-      </c>
-      <c r="E10" s="26">
+      <c r="D10" s="21">
+        <v>30</v>
+      </c>
+      <c r="E10" s="21">
         <v>29.8</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="21">
         <v>29.7</v>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="22">
         <v>117.9</v>
       </c>
       <c r="H10">
-        <f>G10/COUNTIF(C10:F10,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.475000000000001</v>
       </c>
       <c r="I10">
-        <f>H10/3</f>
+        <f t="shared" si="1"/>
+        <v>9.8250000000000011</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="13">
+      <c r="A11" s="12">
         <v>10</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="21">
         <v>27.7</v>
       </c>
-      <c r="D11" s="26">
-        <v>30</v>
-      </c>
-      <c r="E11" s="26">
+      <c r="D11" s="21">
+        <v>30</v>
+      </c>
+      <c r="E11" s="21">
         <v>29.8</v>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="21">
         <v>29.8</v>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="22">
         <v>117.3</v>
       </c>
       <c r="H11">
-        <f>G11/COUNTIF(C11:F11,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.324999999999999</v>
       </c>
       <c r="I11">
-        <f>H11/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7750000000000004</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="13">
+      <c r="A12" s="12">
         <v>11</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="21">
         <v>29.3</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="21">
         <v>29.6</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="21">
         <v>28.3</v>
       </c>
-      <c r="F12" s="26">
+      <c r="F12" s="21">
         <v>29.7</v>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="22">
         <v>116.9</v>
       </c>
       <c r="H12">
-        <f>G12/COUNTIF(C12:F12,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.225000000000001</v>
       </c>
       <c r="I12">
-        <f>H12/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7416666666666671</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13">
+      <c r="A13" s="12">
         <v>12</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="21">
         <v>28.3</v>
       </c>
-      <c r="D13" s="26">
-        <v>30</v>
-      </c>
-      <c r="E13" s="26">
+      <c r="D13" s="21">
+        <v>30</v>
+      </c>
+      <c r="E13" s="21">
         <v>28.8</v>
       </c>
-      <c r="F13" s="26">
+      <c r="F13" s="21">
         <v>29.4</v>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="22">
         <v>116.5</v>
       </c>
       <c r="H13">
-        <f>G13/COUNTIF(C13:F13,"&lt;&gt;0")</f>
+        <f t="shared" si="0"/>
+        <v>29.125</v>
       </c>
       <c r="I13">
-        <f>H13/3</f>
+        <f t="shared" si="1"/>
+        <v>9.7083333333333339</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13">
+      <c r="A14" s="12">
         <v>13</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="21">
         <v>27.5</v>
       </c>
-      <c r="D14" s="26">
-        <v>0</v>
-      </c>
-      <c r="E14" s="26">
+      <c r="D14" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="21">
         <v>29.1</v>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="21">
         <v>29.6</v>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="22">
         <v>86.2</v>
       </c>
       <c r="H14">
-        <f>G14/COUNTIF(C14:F14,"&lt;&gt;0")</f>
+        <f>G14/3</f>
+        <v>28.733333333333334</v>
       </c>
       <c r="I14">
-        <f>H14/3</f>
+        <f t="shared" si="1"/>
+        <v>9.5777777777777775</v>
       </c>
     </row>
   </sheetData>

</xml_diff>